<commit_message>
Update property address in excel
</commit_message>
<xml_diff>
--- a/src/data/properties.xlsx
+++ b/src/data/properties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h2oontherock8\Projects\alexyaphomes\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5D74E83-75FE-408F-B58F-BE308A074E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5DFA30-EDAB-487F-BFB9-6203F1237B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11330" yWindow="2340" windowWidth="26980" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6570" yWindow="2700" windowWidth="26980" windowHeight="17510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="205">
   <si>
     <t>status</t>
   </si>
@@ -202,9 +202,6 @@
   </si>
   <si>
     <t>CA</t>
-  </si>
-  <si>
-    <t>5678 Montalvo Ridge</t>
   </si>
   <si>
     <t>image-01</t>
@@ -653,6 +650,12 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>55 E Hamilton Ave</t>
+  </si>
+  <si>
+    <t>Campbell</t>
   </si>
 </sst>
 </file>
@@ -824,7 +827,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1165,7 +1168,7 @@
   <sheetData>
     <row r="1" spans="1:117" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1192,328 +1195,328 @@
         <v>7</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="O1" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="R1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="S1" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="X1" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="Y1" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="Y1" s="13" t="s">
+      <c r="Z1" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="AA1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="AA1" s="13" t="s">
+      <c r="AB1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AC1" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="AC1" s="13" t="s">
+      <c r="AD1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="AD1" s="13" t="s">
+      <c r="AE1" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="AE1" s="13" t="s">
+      <c r="AF1" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="AF1" s="13" t="s">
+      <c r="AG1" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="AG1" s="13" t="s">
+      <c r="AH1" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="AH1" s="13" t="s">
+      <c r="AI1" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="AI1" s="13" t="s">
+      <c r="AJ1" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="AJ1" s="13" t="s">
+      <c r="AK1" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="AK1" s="13" t="s">
+      <c r="AL1" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="AL1" s="13" t="s">
+      <c r="AM1" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="AM1" s="13" t="s">
+      <c r="AN1" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="AN1" s="13" t="s">
+      <c r="AO1" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="AO1" s="13" t="s">
+      <c r="AP1" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="AP1" s="13" t="s">
+      <c r="AQ1" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="AQ1" s="13" t="s">
+      <c r="AR1" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="AR1" s="13" t="s">
+      <c r="AS1" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="13" t="s">
+      <c r="AT1" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="AT1" s="13" t="s">
+      <c r="AU1" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="AU1" s="13" t="s">
+      <c r="AV1" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="AV1" s="13" t="s">
+      <c r="AW1" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="AW1" s="13" t="s">
+      <c r="AX1" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="AX1" s="13" t="s">
+      <c r="AY1" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="AY1" s="13" t="s">
+      <c r="AZ1" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="AZ1" s="13" t="s">
+      <c r="BA1" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="BA1" s="13" t="s">
+      <c r="BB1" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="BB1" s="13" t="s">
+      <c r="BC1" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="BC1" s="13" t="s">
+      <c r="BD1" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="BD1" s="13" t="s">
+      <c r="BE1" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="BE1" s="13" t="s">
+      <c r="BF1" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="BF1" s="13" t="s">
+      <c r="BG1" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="BG1" s="13" t="s">
+      <c r="BH1" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="BH1" s="13" t="s">
+      <c r="BI1" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="BI1" s="13" t="s">
+      <c r="BJ1" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="BJ1" s="13" t="s">
+      <c r="BK1" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="BK1" s="13" t="s">
+      <c r="BL1" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="BL1" s="13" t="s">
+      <c r="BM1" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="BM1" s="13" t="s">
+      <c r="BN1" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="BN1" s="13" t="s">
+      <c r="BO1" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="BO1" s="13" t="s">
+      <c r="BP1" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="BP1" s="13" t="s">
+      <c r="BQ1" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="BQ1" s="13" t="s">
+      <c r="BR1" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="BR1" s="13" t="s">
+      <c r="BS1" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="BS1" s="13" t="s">
+      <c r="BT1" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="BT1" s="13" t="s">
+      <c r="BU1" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="BU1" s="13" t="s">
+      <c r="BV1" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="BV1" s="13" t="s">
+      <c r="BW1" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="BW1" s="13" t="s">
+      <c r="BX1" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="BX1" s="13" t="s">
+      <c r="BY1" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="BY1" s="13" t="s">
+      <c r="BZ1" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="BZ1" s="13" t="s">
+      <c r="CA1" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="CA1" s="13" t="s">
+      <c r="CB1" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="CB1" s="13" t="s">
+      <c r="CC1" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="CC1" s="13" t="s">
+      <c r="CD1" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="CD1" s="13" t="s">
+      <c r="CE1" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="CE1" s="13" t="s">
+      <c r="CF1" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="CF1" s="13" t="s">
+      <c r="CG1" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="CG1" s="13" t="s">
+      <c r="CH1" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="CH1" s="13" t="s">
+      <c r="CI1" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="CI1" s="13" t="s">
+      <c r="CJ1" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="CJ1" s="13" t="s">
+      <c r="CK1" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="CK1" s="13" t="s">
+      <c r="CL1" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="CL1" s="13" t="s">
+      <c r="CM1" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="CM1" s="13" t="s">
+      <c r="CN1" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="CN1" s="13" t="s">
+      <c r="CO1" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="CO1" s="13" t="s">
+      <c r="CP1" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="CP1" s="13" t="s">
+      <c r="CQ1" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="CQ1" s="13" t="s">
+      <c r="CR1" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="CR1" s="13" t="s">
+      <c r="CS1" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="CS1" s="13" t="s">
+      <c r="CT1" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="CT1" s="13" t="s">
+      <c r="CU1" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="CU1" s="13" t="s">
+      <c r="CV1" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="CV1" s="13" t="s">
+      <c r="CW1" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="CW1" s="13" t="s">
+      <c r="CX1" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="CX1" s="13" t="s">
+      <c r="CY1" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="CY1" s="13" t="s">
+      <c r="CZ1" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="CZ1" s="13" t="s">
+      <c r="DA1" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="DA1" s="13" t="s">
+      <c r="DB1" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="DB1" s="13" t="s">
+      <c r="DC1" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="DC1" s="13" t="s">
+      <c r="DD1" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="DD1" s="13" t="s">
+      <c r="DE1" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="DE1" s="13" t="s">
+      <c r="DF1" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="DF1" s="13" t="s">
+      <c r="DG1" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="DG1" s="13" t="s">
+      <c r="DH1" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="DH1" s="13" t="s">
+      <c r="DI1" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="DI1" s="13" t="s">
+      <c r="DJ1" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="DJ1" s="13" t="s">
+      <c r="DK1" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="DK1" s="13" t="s">
+      <c r="DL1" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="DL1" s="13" t="s">
+      <c r="DM1" s="13" t="s">
         <v>156</v>
-      </c>
-      <c r="DM1" s="13" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:117" ht="44" customHeight="1" x14ac:dyDescent="0.35">
@@ -1525,16 +1528,16 @@
         <v>10</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>57</v>
+        <v>203</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>11</v>
+        <v>204</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
+      <c r="F2" s="2">
+        <v>95008</v>
       </c>
       <c r="G2" s="2">
         <v>5</v>
@@ -1552,7 +1555,7 @@
         <v>14850000</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M2" s="2">
         <v>1970</v>
@@ -1565,71 +1568,71 @@
         <v>1st</v>
       </c>
       <c r="P2" s="17" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Q2" s="19" t="str">
         <f>LOWER(SUBSTITUTE(TRIM(C2), " ", "-")&amp;D2&amp;"-"&amp;E2&amp;"-"&amp;F2)</f>
-        <v>5678-montalvo-ridgesaratoga-ca-95070</v>
+        <v>55-e-hamilton-avecampbell-ca-95008</v>
       </c>
       <c r="R2" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="S2" s="14" t="s">
         <v>23</v>
       </c>
       <c r="T2" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="U2" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="V2" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="V2" s="14" t="s">
-        <v>166</v>
-      </c>
       <c r="W2" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="X2" s="14" t="s">
         <v>23</v>
       </c>
       <c r="Y2" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Z2" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="AA2" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="AA2" s="14" t="s">
-        <v>166</v>
-      </c>
       <c r="AB2" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AC2" s="14" t="s">
         <v>23</v>
       </c>
       <c r="AD2" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AE2" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="AF2" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="AF2" s="14" t="s">
-        <v>166</v>
-      </c>
       <c r="AG2" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AH2" s="14" t="s">
         <v>23</v>
       </c>
       <c r="AI2" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AJ2" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="AK2" s="14" t="s">
         <v>165</v>
-      </c>
-      <c r="AK2" s="14" t="s">
-        <v>166</v>
       </c>
       <c r="AL2" s="14"/>
       <c r="AM2" s="14"/>
@@ -1746,7 +1749,7 @@
         <v>12500000</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M3" s="5">
         <v>1980</v>
@@ -1762,7 +1765,7 @@
         <v>81-bear-creek-ridgelos gatos-ca-95033</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="S3" s="15"/>
       <c r="T3" s="15"/>
@@ -1898,7 +1901,7 @@
         <v>9200000</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="2">
         <v>1960</v>
@@ -1914,7 +1917,7 @@
         <v>330-via-santa-teresamonte sereno-ca-95030</v>
       </c>
       <c r="R4" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="S4" s="14" t="s">
         <v>39</v>
@@ -2052,7 +2055,7 @@
         <v>7400000</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M5" s="5">
         <v>1931</v>
@@ -2070,13 +2073,13 @@
         <v>3271-silver-creek-vistasan jose-ca-95138</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S5" s="15" t="s">
         <v>41</v>
       </c>
       <c r="T5" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U5" s="15"/>
       <c r="V5" s="15"/>
@@ -2210,7 +2213,7 @@
         <v>16750000</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M6" s="2">
         <v>1990</v>
@@ -2228,16 +2231,16 @@
         <v>5045-crescent-park-manorpalo alto-ca-94301</v>
       </c>
       <c r="R6" s="14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="S6" s="14" t="s">
         <v>13</v>
       </c>
       <c r="T6" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U6" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="V6" s="14"/>
       <c r="W6" s="14"/>
@@ -2370,7 +2373,7 @@
         <v>6900000</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M7" s="5">
         <v>2001</v>
@@ -2388,19 +2391,19 @@
         <v>3044-almaden-country-clubsan jose-ca-95120</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="S7" s="15" t="s">
         <v>18</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U7" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="V7" s="15" t="s">
         <v>174</v>
-      </c>
-      <c r="V7" s="15" t="s">
-        <v>175</v>
       </c>
       <c r="W7" s="15"/>
       <c r="X7" s="15"/>
@@ -2532,7 +2535,7 @@
         <v>11200000</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M8" s="2">
         <v>2006</v>
@@ -2548,64 +2551,64 @@
         <v>14550-big-basin-waysaratoga-ca-95070</v>
       </c>
       <c r="R8" s="14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="S8" s="14" t="s">
         <v>23</v>
       </c>
       <c r="T8" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="U8" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="V8" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="V8" s="14" t="s">
-        <v>176</v>
-      </c>
       <c r="W8" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="X8" s="14" t="s">
         <v>23</v>
       </c>
       <c r="Y8" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Z8" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA8" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="AA8" s="14" t="s">
-        <v>176</v>
-      </c>
       <c r="AB8" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AC8" s="14" t="s">
         <v>23</v>
       </c>
       <c r="AD8" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AE8" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="AF8" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="AF8" s="14" t="s">
-        <v>176</v>
-      </c>
       <c r="AG8" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AH8" s="14" t="s">
         <v>23</v>
       </c>
       <c r="AI8" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AJ8" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="AK8" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="AK8" s="14" t="s">
-        <v>176</v>
       </c>
       <c r="AL8" s="14"/>
       <c r="AM8" s="14"/>
@@ -2722,7 +2725,7 @@
         <v>8650000</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M9" s="5">
         <v>2021</v>
@@ -2738,64 +2741,64 @@
         <v>210-shannon-roadlos gatos-ca-95032</v>
       </c>
       <c r="R9" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="S9" s="15" t="s">
         <v>27</v>
       </c>
       <c r="T9" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="U9" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="V9" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="V9" s="15" t="s">
-        <v>177</v>
-      </c>
       <c r="W9" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="X9" s="15" t="s">
         <v>27</v>
       </c>
       <c r="Y9" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Z9" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA9" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="AA9" s="15" t="s">
-        <v>177</v>
-      </c>
       <c r="AB9" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AC9" s="15" t="s">
         <v>27</v>
       </c>
       <c r="AD9" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AE9" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="AF9" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="AF9" s="15" t="s">
-        <v>177</v>
-      </c>
       <c r="AG9" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AH9" s="15" t="s">
         <v>27</v>
       </c>
       <c r="AI9" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ9" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="AK9" s="15" t="s">
         <v>176</v>
-      </c>
-      <c r="AK9" s="15" t="s">
-        <v>177</v>
       </c>
       <c r="AL9" s="15"/>
       <c r="AM9" s="15"/>
@@ -2912,7 +2915,7 @@
         <v>13800000</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M10" s="2">
         <v>1945</v>
@@ -2928,64 +2931,64 @@
         <v>16200-greenwood-lanemonte sereno-ca-95030</v>
       </c>
       <c r="R10" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="S10" s="14" t="s">
         <v>31</v>
       </c>
       <c r="T10" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="U10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="V10" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="U10" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="V10" s="14" t="s">
-        <v>176</v>
-      </c>
       <c r="W10" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="X10" s="14" t="s">
         <v>31</v>
       </c>
       <c r="Y10" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="Z10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AA10" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="Z10" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA10" s="14" t="s">
-        <v>176</v>
-      </c>
       <c r="AB10" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AC10" s="14" t="s">
         <v>31</v>
       </c>
       <c r="AD10" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="AE10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF10" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="AE10" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="AF10" s="14" t="s">
-        <v>176</v>
-      </c>
       <c r="AG10" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AH10" s="14" t="s">
         <v>31</v>
       </c>
       <c r="AI10" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="AJ10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AK10" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="AJ10" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="AK10" s="14" t="s">
-        <v>176</v>
       </c>
       <c r="AL10" s="14"/>
       <c r="AM10" s="14"/>
@@ -3102,7 +3105,7 @@
         <v>7950000</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M11" s="5">
         <v>1950</v>
@@ -3118,64 +3121,64 @@
         <v>389-university-avenuelos altos-ca-94022</v>
       </c>
       <c r="R11" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="S11" s="15" t="s">
         <v>34</v>
       </c>
       <c r="T11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="V11" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="W11" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="X11" s="15" t="s">
         <v>34</v>
       </c>
       <c r="Y11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Z11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AA11" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB11" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AC11" s="15" t="s">
         <v>34</v>
       </c>
       <c r="AD11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AE11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AF11" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AG11" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AH11" s="15" t="s">
         <v>34</v>
       </c>
       <c r="AI11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AJ11" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AK11" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AL11" s="15"/>
       <c r="AM11" s="15"/>
@@ -3292,7 +3295,7 @@
         <v>15200000</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M12" s="2">
         <v>1940</v>
@@ -3308,64 +3311,64 @@
         <v>1050-waverley-streetpalo alto-ca-94301</v>
       </c>
       <c r="R12" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="S12" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T12" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="U12" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="U12" s="14" t="s">
+      <c r="V12" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="V12" s="14" t="s">
-        <v>179</v>
-      </c>
       <c r="W12" s="14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="X12" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Y12" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z12" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="Z12" s="14" t="s">
+      <c r="AA12" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="AA12" s="14" t="s">
-        <v>179</v>
-      </c>
       <c r="AB12" s="14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AC12" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AD12" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AE12" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="AE12" s="14" t="s">
+      <c r="AF12" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="AF12" s="14" t="s">
-        <v>179</v>
-      </c>
       <c r="AG12" s="14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AH12" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AI12" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AJ12" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="AJ12" s="14" t="s">
+      <c r="AK12" s="14" t="s">
         <v>178</v>
-      </c>
-      <c r="AK12" s="14" t="s">
-        <v>179</v>
       </c>
       <c r="AL12" s="14"/>
       <c r="AM12" s="14"/>
@@ -3482,7 +3485,7 @@
         <v>6450000</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M13" s="5">
         <v>1931</v>
@@ -3498,64 +3501,64 @@
         <v>6220-country-club-pkwysan jose-ca-95138</v>
       </c>
       <c r="R13" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="S13" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U13" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="V13" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="V13" s="15" t="s">
-        <v>180</v>
-      </c>
       <c r="W13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="X13" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Y13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Z13" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="AA13" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="AA13" s="15" t="s">
-        <v>180</v>
-      </c>
       <c r="AB13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AC13" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AD13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AE13" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="AF13" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="AF13" s="15" t="s">
-        <v>180</v>
-      </c>
       <c r="AG13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AH13" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AI13" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AJ13" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="AK13" s="15" t="s">
         <v>179</v>
-      </c>
-      <c r="AK13" s="15" t="s">
-        <v>180</v>
       </c>
       <c r="AL13" s="15"/>
       <c r="AM13" s="15"/>
@@ -3672,7 +3675,7 @@
         <v>10950000</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M14" s="2">
         <v>1950</v>
@@ -3688,64 +3691,64 @@
         <v>19540-glen-una-drivesaratoga-ca-95070</v>
       </c>
       <c r="R14" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="S14" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T14" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U14" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="V14" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="14" t="s">
-        <v>181</v>
-      </c>
       <c r="W14" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="X14" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y14" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="X14" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="Y14" s="14" t="s">
-        <v>178</v>
-      </c>
       <c r="Z14" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="AA14" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="AA14" s="14" t="s">
-        <v>181</v>
-      </c>
       <c r="AB14" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AC14" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="AD14" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="AC14" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="AD14" s="14" t="s">
-        <v>178</v>
-      </c>
       <c r="AE14" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="AF14" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="AF14" s="14" t="s">
-        <v>181</v>
-      </c>
       <c r="AG14" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AH14" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="AI14" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="AH14" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="AI14" s="14" t="s">
-        <v>178</v>
-      </c>
       <c r="AJ14" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="AK14" s="14" t="s">
         <v>180</v>
-      </c>
-      <c r="AK14" s="14" t="s">
-        <v>181</v>
       </c>
       <c r="AL14" s="14"/>
       <c r="AM14" s="14"/>
@@ -3862,7 +3865,7 @@
         <v>5850000</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M15" s="5">
         <v>1960</v>
@@ -3878,64 +3881,64 @@
         <v>15420-francis-oaks-waylos gatos-ca-95032</v>
       </c>
       <c r="R15" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="S15" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T15" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U15" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="V15" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="15" t="s">
-        <v>182</v>
-      </c>
       <c r="W15" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="X15" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Y15" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Z15" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="AA15" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="AA15" s="15" t="s">
-        <v>182</v>
-      </c>
       <c r="AB15" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AC15" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AD15" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AE15" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="AF15" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="AF15" s="15" t="s">
-        <v>182</v>
-      </c>
       <c r="AG15" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AH15" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI15" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AJ15" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="AK15" s="15" t="s">
         <v>181</v>
-      </c>
-      <c r="AK15" s="15" t="s">
-        <v>182</v>
       </c>
       <c r="AL15" s="15"/>
       <c r="AM15" s="15"/>
@@ -4052,7 +4055,7 @@
         <v>5200000</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M16" s="2">
         <v>1951</v>
@@ -4068,64 +4071,64 @@
         <v>18230-daves-avenuemonte sereno-ca-95030</v>
       </c>
       <c r="R16" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="S16" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T16" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U16" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="V16" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="V16" s="14" t="s">
-        <v>183</v>
-      </c>
       <c r="W16" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="X16" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="Y16" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Z16" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA16" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="AA16" s="14" t="s">
-        <v>183</v>
-      </c>
       <c r="AB16" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AC16" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AD16" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AE16" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="AF16" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="AF16" s="14" t="s">
-        <v>183</v>
-      </c>
       <c r="AG16" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AH16" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AI16" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AJ16" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK16" s="14" t="s">
         <v>182</v>
-      </c>
-      <c r="AK16" s="14" t="s">
-        <v>183</v>
       </c>
       <c r="AL16" s="14"/>
       <c r="AM16" s="14"/>
@@ -4242,7 +4245,7 @@
         <v>12900000</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M17" s="5">
         <v>2023</v>
@@ -4258,64 +4261,64 @@
         <v>23000-congress-springs-rdsaratoga-ca-95070</v>
       </c>
       <c r="R17" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="S17" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T17" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U17" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V17" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="W17" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="X17" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Y17" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Z17" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AA17" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AB17" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AC17" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AD17" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AE17" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AF17" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AG17" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AH17" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AI17" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AJ17" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AK17" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AL17" s="15"/>
       <c r="AM17" s="15"/>
@@ -4432,7 +4435,7 @@
         <v>9400000</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M18" s="2">
         <v>1997</v>
@@ -4448,64 +4451,64 @@
         <v>750-university-avenuelos altos-ca-94022</v>
       </c>
       <c r="R18" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="S18" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="U18" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="V18" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="V18" s="14" t="s">
-        <v>162</v>
-      </c>
       <c r="W18" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="X18" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Y18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z18" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="AA18" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="AA18" s="14" t="s">
-        <v>162</v>
-      </c>
       <c r="AB18" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AC18" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AD18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE18" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="AF18" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="AF18" s="14" t="s">
-        <v>162</v>
-      </c>
       <c r="AG18" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AH18" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AI18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AJ18" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="AK18" s="14" t="s">
         <v>161</v>
-      </c>
-      <c r="AK18" s="14" t="s">
-        <v>162</v>
       </c>
       <c r="AL18" s="14"/>
       <c r="AM18" s="14"/>
@@ -4622,7 +4625,7 @@
         <v>6150000</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M19" s="5">
         <v>1994</v>
@@ -4638,64 +4641,64 @@
         <v>16100-kennedy-roadlos gatos-ca-95032</v>
       </c>
       <c r="R19" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="S19" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="T19" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="U19" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="V19" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="V19" s="15" t="s">
-        <v>163</v>
-      </c>
       <c r="W19" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="X19" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Y19" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z19" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="AA19" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="AA19" s="15" t="s">
-        <v>163</v>
-      </c>
       <c r="AB19" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AC19" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AD19" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AE19" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="AF19" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="AF19" s="15" t="s">
-        <v>163</v>
-      </c>
       <c r="AG19" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AH19" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AI19" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AJ19" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="AK19" s="15" t="s">
         <v>162</v>
-      </c>
-      <c r="AK19" s="15" t="s">
-        <v>163</v>
       </c>
       <c r="AL19" s="15"/>
       <c r="AM19" s="15"/>
@@ -4812,7 +4815,7 @@
         <v>5750000</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M20" s="2">
         <v>1980</v>
@@ -4828,64 +4831,64 @@
         <v>21540-almaden-roadsan jose-ca-95120</v>
       </c>
       <c r="R20" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="S20" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="T20" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="U20" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="V20" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="V20" s="14" t="s">
-        <v>164</v>
-      </c>
       <c r="W20" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="X20" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Y20" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Z20" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="AA20" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="AA20" s="14" t="s">
-        <v>164</v>
-      </c>
       <c r="AB20" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC20" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AD20" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AE20" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="AF20" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="AF20" s="14" t="s">
-        <v>164</v>
-      </c>
       <c r="AG20" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH20" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AI20" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AJ20" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="AK20" s="14" t="s">
         <v>163</v>
-      </c>
-      <c r="AK20" s="14" t="s">
-        <v>164</v>
       </c>
       <c r="AL20" s="14"/>
       <c r="AM20" s="14"/>
@@ -5002,7 +5005,7 @@
         <v>6800000</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M21" s="5">
         <v>1951</v>
@@ -5018,64 +5021,64 @@
         <v>4120-miranda-avenuepalo alto-ca-94306</v>
       </c>
       <c r="R21" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="S21" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T21" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="U21" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="V21" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="V21" s="15" t="s">
-        <v>165</v>
-      </c>
       <c r="W21" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X21" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Y21" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Z21" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="AA21" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="AA21" s="15" t="s">
-        <v>165</v>
-      </c>
       <c r="AB21" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AC21" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AD21" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AE21" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="AF21" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="AF21" s="15" t="s">
-        <v>165</v>
-      </c>
       <c r="AG21" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AH21" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AI21" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AJ21" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="AK21" s="15" t="s">
         <v>164</v>
-      </c>
-      <c r="AK21" s="15" t="s">
-        <v>165</v>
       </c>
       <c r="AL21" s="15"/>
       <c r="AM21" s="15"/>

</xml_diff>